<commit_message>
fix: correct Novelia Harlinda NIM to 24050530045 across database, README, and Excel workbooks
</commit_message>
<xml_diff>
--- a/DRIVE MASTER NIRANTARA PLK UNY 2027/01_KESEKRETARIATAN/03_Logbook_272_Jam/Master_Logbook_272_Jam_Kerja.xlsx
+++ b/DRIVE MASTER NIRANTARA PLK UNY 2027/01_KESEKRETARIATAN/03_Logbook_272_Jam/Master_Logbook_272_Jam_Kerja.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>24520244xxx</t>
+          <t>24050530030</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>24520244xxx</t>
+          <t>24050530052</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -685,7 +685,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>24520244xxx</t>
+          <t>24050530029</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>24520244xxx</t>
+          <t>24050530045</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>24802241xxx</t>
+          <t>24080330053</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>24802241xxx</t>
+          <t>24080330078</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>24308144xxx</t>
+          <t>24030830059</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>24308144xxx</t>
+          <t>24030830068</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>24105244xxx</t>
+          <t>24010530018</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>24105244xxx</t>
+          <t>24010530004</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">

</xml_diff>